<commit_message>
Add Korea grid-mix abatement cases to scale-up report section 4
- section 4: added KRmix WTWa GHG rows and a Korea-method abatement table
  (full-ammonia + full-CCS, T&S range) alongside the U.S. tables; corrected the
  prior mislabel (existing tables were U.S., not KR). Korea grid raises CCS
  abatement ~6% (base scale alloc 460/674 vs U.S. 433/635); ammonia unchanged.
- tea_scale_up_abatement.py: reads GHG-100 from Pyrolysis_551_LCA_*_KRmix via
  funs_lca.get_WTWa_pyrolysis and emits Korea full-option abatement per scale.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MjFwwDgUpjrZDZMd1ma7x
</commit_message>
<xml_diff>
--- a/Figure/scale_up_abatement.xlsx
+++ b/Figure/scale_up_abatement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS8"/>
+  <dimension ref="A1:AY8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -654,6 +654,36 @@
           <t>CCS100_abate_disp_ts0</t>
         </is>
       </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Amm_KRalloc</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Amm_KRdisp</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>CCS100_KRalloc_ts4</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>CCS100_KRdisp_ts4</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>CCS100_KRalloc_ts45</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>CCS100_KRdisp_ts45</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -791,6 +821,24 @@
       <c r="AS2" t="n">
         <v>130.519</v>
       </c>
+      <c r="AT2" t="n">
+        <v>1529.219</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>482.185</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>460.322</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>145.165</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>674.477</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>212.7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -928,6 +976,24 @@
       <c r="AS3" t="n">
         <v>120.893</v>
       </c>
+      <c r="AT3" t="n">
+        <v>1485.484</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>468.395</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>427.914</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>134.945</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>642.068</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>202.479</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -1065,6 +1131,24 @@
       <c r="AS4" t="n">
         <v>115.628</v>
       </c>
+      <c r="AT4" t="n">
+        <v>1471.184</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>463.886</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>410.188</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>129.355</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>624.342</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>196.889</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1202,6 +1286,24 @@
       <c r="AS5" t="n">
         <v>113.161</v>
       </c>
+      <c r="AT5" t="n">
+        <v>1463.183</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>461.363</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>401.881</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>126.735</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>616.0359999999999</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>194.27</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1339,6 +1441,24 @@
       <c r="AS6" t="n">
         <v>111.638</v>
       </c>
+      <c r="AT6" t="n">
+        <v>1452.325</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>457.939</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>396.754</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>125.118</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>610.908</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>192.653</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -1476,6 +1596,24 @@
       <c r="AS7" t="n">
         <v>108.614</v>
       </c>
+      <c r="AT7" t="n">
+        <v>1434.312</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>452.259</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>386.572</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>121.907</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>600.727</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>189.442</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1612,6 +1750,24 @@
       </c>
       <c r="AS8" t="n">
         <v>107.197</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1430.426</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>451.034</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>381.802</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>120.403</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>595.956</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>187.938</v>
       </c>
     </row>
   </sheetData>

</xml_diff>